<commit_message>
Removed HtmlReports from Git tracking
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDataFile/TestData.xlsx
+++ b/src/test/resources/TestDataFile/TestData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t>Testname</t>
   </si>
@@ -52,6 +52,12 @@
   <si>
     <t>Power Bank</t>
   </si>
+  <si>
+    <t>Test3</t>
+  </si>
+  <si>
+    <t>https://www.worldometers.info/coronavirus/#main_table</t>
+  </si>
 </sst>
 </file>
 
@@ -85,18 +91,18 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -539,28 +545,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -684,10 +690,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1163,10 +1170,10 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="12.6285714285714" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="2" outlineLevelCol="2"/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="12.6285714285714" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="3" outlineLevelCol="2"/>
   <cols>
-    <col min="2" max="2" width="38.5047619047619" customWidth="1"/>
+    <col min="2" max="2" width="42.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:3">
@@ -1202,7 +1209,18 @@
         <v>7</v>
       </c>
     </row>
+    <row r="4" customHeight="1" spans="1:2">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" display="https://www.worldometers.info/coronavirus/#main_table" tooltip="https://www.worldometers.info/coronavirus/#main_table"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>